<commit_message>
fix(hospital): xlsx-lite dropped cells after a self-closing empty cell (column misalign)
The real root cause behind both the cédula-mapping skew AND the collapsed
hospitalizado count: xlsx-lite's per-cell regex matched the open/close form before
the self-closing form, so a greedy open-tag branch swallowed the cell AFTER a
self-closing empty cell (`<c r="F5"/>`). Rows with an empty middle column (very
common — blank teléfono/dirección) lost their OBSERVACIONES → parsed as
'desconocido' instead of 'hospitalizado', and columns shifted.

Fix: one non-greedy regex per cell with a `(?:/>|>…</c>)` alternation that matches a
self-closing cell first. Verified on the real 7,431-row file: estado now
hospitalizado 4,111 / alta 656 / fallecido 95 / desconocido 2,568 (was 1,262 /
5,532 before), matching openpyxl. Regression fixture now includes gappy rows.
Full suite green.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/fixtures/hospital-sample.xlsx
+++ b/test/fixtures/hospital-sample.xlsx
@@ -426,7 +426,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>info</t>
+          <t>Actualizado: 30JUN26 00:40h</t>
         </is>
       </c>
     </row>
@@ -538,9 +538,6 @@
           <t>50</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Alta médica</t>
@@ -566,9 +563,6 @@
           <t>36</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>FALLECIDO | ⚠ ESTADO EN CONFLICTO</t>

</xml_diff>